<commit_message>
I modified the dashboard
</commit_message>
<xml_diff>
--- a/data/HR_Analytics_Capstone_Raw_Data.xlsx
+++ b/data/HR_Analytics_Capstone_Raw_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\IOTBTECH 2026\Excel Folder\Excel-Capstone-Project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{464D043E-385C-4EA5-BFC7-4C2AA504AB00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA1E6B5-8E15-4898-97CB-DA2D8495374C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Analysis" sheetId="6" r:id="rId1"/>
@@ -28,7 +28,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId8"/>
+    <pivotCache cacheId="2" r:id="rId8"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -983,13 +983,13 @@
     <t>Total_Bonus</t>
   </si>
   <si>
-    <t>Average of Year_of_Service</t>
+    <t>Average Year_of_Service</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
@@ -1007,6 +1007,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1131,225 +1132,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="86">
+  <dxfs count="26">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="166" formatCode="&quot;₦&quot;#,##0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="13" formatCode="0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1397,24 +1188,99 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;₦&quot;#,##0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <sz val="11"/>
+        <color auto="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <gradientFill degree="90">
+          <stop position="0">
+            <color theme="4"/>
+          </stop>
+          <stop position="1">
+            <color rgb="FF4F81BD"/>
+          </stop>
+        </gradientFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <sz val="12"/>
+        <color rgb="FF31859C"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="11"/>
+        <color rgb="FF4F81BD"/>
+      </font>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="4" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Slicer Style 1" pivot="0" table="0" count="1" xr9:uid="{F1B4E4D4-7881-425E-8960-774055D62EEF}">
+      <tableStyleElement type="wholeTable" dxfId="25"/>
+    </tableStyle>
+    <tableStyle name="Slicer Style 2" pivot="0" table="0" count="0" xr9:uid="{5556B23E-21AB-4165-85A7-BBBBFA797A00}"/>
+    <tableStyle name="Slicer Style 3" pivot="0" table="0" count="1" xr9:uid="{E0ACD3C2-6CF8-4BAC-BD3A-F7DF1EBD72B3}">
+      <tableStyleElement type="wholeTable" dxfId="24"/>
+    </tableStyle>
+    <tableStyle name="Slicer Style 4" pivot="0" table="0" count="2" xr9:uid="{16AC44C9-1B35-4F01-9F91-B5681BCDA9F7}">
+      <tableStyleElement type="wholeTable" dxfId="23"/>
+      <tableStyleElement type="headerRow" dxfId="22"/>
+    </tableStyle>
+  </tableStyles>
   <colors>
     <mruColors>
+      <color rgb="FF4F81BD"/>
+      <color rgb="FF31859C"/>
       <color rgb="FFDBEEF4"/>
       <color rgb="FF000000"/>
-      <color rgb="FF31859C"/>
-      <color rgb="FF4F81BD"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1">
+        <x14:slicerStyle name="Slicer Style 1"/>
+        <x14:slicerStyle name="Slicer Style 2"/>
+        <x14:slicerStyle name="Slicer Style 3"/>
+        <x14:slicerStyle name="Slicer Style 4"/>
+      </x14:slicerStyles>
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
       <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
@@ -4286,7 +4152,6 @@
               <a:endParaRPr lang="en-NG"/>
             </a:p>
           </c:txPr>
-          <c:dLblPos val="inEnd"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -4378,7 +4243,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="inEnd"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -10318,7 +10182,7 @@
 </file>
 
 <file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="21">
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
   <a:schemeClr val="accent1"/>
 </cs:colorStyle>
 </file>
@@ -15669,89 +15533,6 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>867833</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>29633</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>92075</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="10" name="Performance_Band">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCECD390-2B26-96E6-7E96-AD5F3C778687}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Performance_Band"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="9080500" y="1949450"/>
-              <a:ext cx="1828800" cy="2524125"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-NG" sz="1100"/>
-                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
-If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -15983,7 +15764,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -16088,9 +15869,7 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="31859C">
-            <a:alpha val="20000"/>
-          </a:srgbClr>
+          <a:srgbClr val="31859C"/>
         </a:solidFill>
         <a:ln>
           <a:noFill/>
@@ -16202,9 +15981,7 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="31859C">
-            <a:alpha val="20000"/>
-          </a:srgbClr>
+          <a:srgbClr val="31859C"/>
         </a:solidFill>
         <a:ln>
           <a:solidFill>
@@ -16252,18 +16029,19 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>317505</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>31738</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>82538</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>198441</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>15864</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>66664</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="8" name="Rectangle: Rounded Corners 7">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA0A922B-C5A9-4DEA-AE7D-369A4C1242F2}"/>
@@ -16274,8 +16052,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="317505" y="2039926"/>
-          <a:ext cx="1714499" cy="531813"/>
+          <a:off x="317505" y="2368538"/>
+          <a:ext cx="1709736" cy="555626"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
@@ -16355,6 +16133,7 @@
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="10" name="Rectangle: Rounded Corners 9">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CCC946EB-CB39-478A-A94E-22CCE55BAAA5}"/>
@@ -16434,18 +16213,19 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>309563</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>63500</xdr:rowOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>190499</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>187325</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="12" name="Rectangle: Rounded Corners 11">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{373ABAFA-A904-4274-980E-088124BB58A3}"/>
@@ -16456,15 +16236,15 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="309563" y="2984500"/>
-          <a:ext cx="1714499" cy="531813"/>
+          <a:off x="309563" y="3632200"/>
+          <a:ext cx="1709736" cy="555625"/>
         </a:xfrm>
         <a:prstGeom prst="roundRect">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
           <a:srgbClr val="31859C">
-            <a:alpha val="20000"/>
+            <a:alpha val="89804"/>
           </a:srgbClr>
         </a:solidFill>
         <a:ln>
@@ -17440,6 +17220,17 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+              <a:ea typeface="Calibri"/>
+              <a:cs typeface="Calibri"/>
+            </a:rPr>
+            <a:t>              </a:t>
+          </a:r>
           <a:fld id="{97DCB790-AC7E-4E45-AD19-199BF919F77C}" type="TxLink">
             <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
@@ -17449,6 +17240,7 @@
               <a:ea typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr algn="l"/>
             <a:t>150</a:t>
           </a:fld>
           <a:endParaRPr lang="en-NG" sz="1100"/>
@@ -17535,6 +17327,7 @@
               <a:ea typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr algn="l"/>
             <a:t>₦506,179.88</a:t>
           </a:fld>
           <a:endParaRPr lang="en-NG" sz="1100"/>
@@ -17621,6 +17414,7 @@
               <a:ea typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr algn="l"/>
             <a:t>22%</a:t>
           </a:fld>
           <a:endParaRPr lang="en-NG" sz="1100"/>
@@ -17707,6 +17501,7 @@
               <a:ea typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr algn="l"/>
             <a:t>₦496,463.30</a:t>
           </a:fld>
           <a:endParaRPr lang="en-NG" sz="1100"/>
@@ -17793,6 +17588,7 @@
               <a:ea typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
+            <a:pPr algn="l"/>
             <a:t>6.44</a:t>
           </a:fld>
           <a:endParaRPr lang="en-NG" sz="1100"/>
@@ -18141,7 +17937,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -18179,7 +17975,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -18217,7 +18013,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -18255,7 +18051,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -18274,8 +18070,8 @@
       <xdr:row>21</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="45" name="Department_Name 1">
@@ -18298,7 +18094,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -18352,8 +18148,8 @@
       <xdr:row>29</xdr:row>
       <xdr:rowOff>25400</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="46" name="Cleaned Employment_Status 1">
@@ -18376,7 +18172,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -18430,8 +18226,8 @@
       <xdr:row>39</xdr:row>
       <xdr:rowOff>165101</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="47" name="Performance_Band 1">
@@ -18454,7 +18250,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -20978,7 +20774,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F4E7B9D-DDA8-4061-9C46-C8585D2A937B}" name="PivotTable8" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="30" rowHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F4E7B9D-DDA8-4061-9C46-C8585D2A937B}" name="PivotTable8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="30" rowHeaderCaption="">
   <location ref="F28:F29" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -21020,16 +20816,16 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Average of Year_of_Service" fld="7" subtotal="average" baseField="0" baseItem="0"/>
+    <dataField name="Average Year_of_Service" fld="7" subtotal="average" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="67">
+    <format dxfId="16">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="66">
+    <format dxfId="15">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="65">
+    <format dxfId="14">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -21046,644 +20842,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6ACE57F1-1121-49BE-A770-63A5C79D6E65}" name="PivotTable6" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="30" rowHeaderCaption="">
-  <location ref="A28:A29" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField dataField="1" numFmtId="9" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowItems count="1">
-    <i/>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Eligible_Bonus_Amount" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="71">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6343A1DA-E553-4739-9DC1-7663658B3C83}" name="PivotTable5" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34" rowHeaderCaption="Department_Name">
-  <location ref="L17:M23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField dataField="1" numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average of Cleaned Salary" fld="8" subtotal="average" baseField="4" baseItem="2" numFmtId="165"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="72">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="29" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="33" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9766C7AF-3425-454D-9C4E-268C288647D8}" name="PivotTable4" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="27" rowHeaderCaption="Department_Name">
-  <location ref="F17:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Head_Count" fld="0" subtotal="count" baseField="4" baseItem="1"/>
-  </dataFields>
-  <chartFormats count="2">
-    <chartFormat chart="22" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="25" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C65AF6F8-97EA-40FE-926F-D435681070FB}" name="PivotTable2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="28" rowHeaderCaption="Performance Band">
-  <location ref="A17:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="1"/>
-        <item x="0"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField dataField="1" numFmtId="9" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="10"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of Eligible_Bonus_Amount" fld="12" baseField="10" baseItem="0" numFmtId="165"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="64">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
-    </format>
-  </formats>
-  <chartFormats count="4">
-    <chartFormat chart="6" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="10" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="24" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="27" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D5CA70F-9904-4A47-AFC0-00D008E6E30C}" name="PivotTable1" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Employment_Status">
-  <location ref="N3:O6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="166" showAll="0"/>
-    <pivotField dataField="1" numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="13"/>
-  </rowFields>
-  <rowItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Average Perf_Score" fld="9" subtotal="average" baseField="12" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="4">
-    <chartFormat chart="13" format="13" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="13" format="14">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="13" format="15">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="13" format="16">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="13" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{95C03F21-8440-4E60-A15F-EDE839858110}" name="Headcount &amp; Average Salary by Department" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Department_Name">
-  <location ref="A3:C9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="7">
-        <item x="2"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField dataField="1" numFmtId="166" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="4"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="2">
-    <dataField name="HeadCount" fld="0" subtotal="count" baseField="4" baseItem="0"/>
-    <dataField name="Average Salary" fld="8" subtotal="average" baseField="4" baseItem="0" numFmtId="165"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="85">
-      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="84">
-      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <chartFormats count="2">
-    <chartFormat chart="6" format="4" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="6" format="5" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FEAA84F8-7B84-44FD-A04F-FD9B3F7229C6}" name="PivotTable3" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12" rowHeaderCaption="Employment_Status">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FEAA84F8-7B84-44FD-A04F-FD9B3F7229C6}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12" rowHeaderCaption="Employment_Status">
   <location ref="F3:G7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -21800,6 +20959,643 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6ACE57F1-1121-49BE-A770-63A5C79D6E65}" name="PivotTable6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="30" rowHeaderCaption="">
+  <location ref="A28:A29" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField dataField="1" numFmtId="9" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Eligible_Bonus_Amount" fld="12" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="17">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9766C7AF-3425-454D-9C4E-268C288647D8}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="38" rowHeaderCaption="Department_Name">
+  <location ref="F17:G23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Head_Count" fld="0" subtotal="count" baseField="4" baseItem="1"/>
+  </dataFields>
+  <chartFormats count="2">
+    <chartFormat chart="22" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="25" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C65AF6F8-97EA-40FE-926F-D435681070FB}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="28" rowHeaderCaption="Performance Band">
+  <location ref="A17:B22" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField dataField="1" numFmtId="9" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="10"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Eligible_Bonus_Amount" fld="12" baseField="10" baseItem="0" numFmtId="165"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="18">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="4">
+    <chartFormat chart="6" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="10" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="24" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="27" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3D5CA70F-9904-4A47-AFC0-00D008E6E30C}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Employment_Status">
+  <location ref="N3:O6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="166" showAll="0"/>
+    <pivotField dataField="1" numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="13"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average Perf_Score" fld="9" subtotal="average" baseField="12" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="4">
+    <chartFormat chart="13" format="13" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="14">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="15">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="13" format="16">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="13" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{95C03F21-8440-4E60-A15F-EDE839858110}" name="Headcount &amp; Average Salary by Department" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Department_Name">
+  <location ref="A3:C9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="2">
+    <dataField name="HeadCount" fld="0" subtotal="count" baseField="4" baseItem="0"/>
+    <dataField name="Average Salary" fld="8" subtotal="average" baseField="4" baseItem="0" numFmtId="165"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="20">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="19">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="6" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="6" format="5" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable8.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6343A1DA-E553-4739-9DC1-7663658B3C83}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34" rowHeaderCaption="Department_Name">
+  <location ref="L17:M23" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="7">
+        <item x="2"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField dataField="1" numFmtId="166" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Cleaned Salary" fld="8" subtotal="average" baseField="4" baseItem="2" numFmtId="165"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="21">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+  </formats>
+  <chartFormats count="2">
+    <chartFormat chart="29" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="33" format="4" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Department_Name" xr10:uid="{3B112148-E306-4B09-8CC8-B4A4C081DB54}" sourceName="Department_Name">
   <pivotTables>
@@ -21872,15 +21668,9 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="Performance_Band" xr10:uid="{2305E51B-059D-4CDE-A801-0D94794A1F7F}" cache="Slicer_Performance_Band" caption="Performance_Band" rowHeight="241300"/>
-</slicers>
-</file>
-
-<file path=xl/slicers/slicer2.xml><?xml version="1.0" encoding="utf-8"?>
-<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="Department_Name 1" xr10:uid="{3057399E-2EEB-4C29-B1CD-3CCD915A91DA}" cache="Slicer_Department_Name" caption="Department_Name" rowHeight="241300"/>
-  <slicer name="Cleaned Employment_Status 1" xr10:uid="{354F92D9-FABC-46C6-8856-75884730C768}" cache="Slicer_Cleaned_Employment_Status" caption="Cleaned Employment_Status" rowHeight="241300"/>
-  <slicer name="Performance_Band 1" xr10:uid="{CD084D95-A3F3-48C8-92C2-C5D09409DB6D}" cache="Slicer_Performance_Band" caption="Performance_Band" rowHeight="241300"/>
+  <slicer name="Department_Name 1" xr10:uid="{3057399E-2EEB-4C29-B1CD-3CCD915A91DA}" cache="Slicer_Department_Name" caption="Department_Name" style="Slicer Style 4" rowHeight="241300"/>
+  <slicer name="Cleaned Employment_Status 1" xr10:uid="{354F92D9-FABC-46C6-8856-75884730C768}" cache="Slicer_Cleaned_Employment_Status" caption="Cleaned Employment_Status" style="Slicer Style 4" rowHeight="241300"/>
+  <slicer name="Performance_Band 1" xr10:uid="{CD084D95-A3F3-48C8-92C2-C5D09409DB6D}" cache="Slicer_Performance_Band" caption="Performance_Band" style="Slicer Style 4" rowHeight="241300"/>
 </slicers>
 </file>
 
@@ -21888,46 +21678,46 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D86B9076-85AF-44F4-9A85-F17D0151F005}" name="Table1" displayName="Table1" ref="J1:W151" totalsRowShown="0">
   <autoFilter ref="J1:W151" xr:uid="{D86B9076-85AF-44F4-9A85-F17D0151F005}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{08AF9922-978B-4E5E-B1AD-14907D7F178F}" name="Cleaned EMP ID" dataDxfId="83">
+    <tableColumn id="1" xr3:uid="{08AF9922-978B-4E5E-B1AD-14907D7F178F}" name="Cleaned EMP ID" dataDxfId="13">
       <calculatedColumnFormula>TRIM(CLEAN(A2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{8CEE1055-2A2F-4DA0-BEB9-363B105F5B43}" name="Cleaned First_Name" dataDxfId="82">
+    <tableColumn id="2" xr3:uid="{8CEE1055-2A2F-4DA0-BEB9-363B105F5B43}" name="Cleaned First_Name" dataDxfId="12">
       <calculatedColumnFormula>TRIM(CLEAN(PROPER(B2)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1BACBA2A-31FA-4BFA-AC56-8B690BBBE17A}" name="Cleaned Last_Name" dataDxfId="81">
+    <tableColumn id="3" xr3:uid="{1BACBA2A-31FA-4BFA-AC56-8B690BBBE17A}" name="Cleaned Last_Name" dataDxfId="11">
       <calculatedColumnFormula>TRIM(CLEAN(PROPER(C2)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{ACDDBD44-DED7-45A0-A91C-C301EA2FC8DF}" name="Full_Name" dataDxfId="80">
+    <tableColumn id="4" xr3:uid="{ACDDBD44-DED7-45A0-A91C-C301EA2FC8DF}" name="Full_Name" dataDxfId="10">
       <calculatedColumnFormula>_xlfn.TEXTJOIN(" ",TRUE,K2,L2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{3ACDA19A-4009-42B7-9CEC-E31BB63C9FF9}" name="Department_Name" dataDxfId="79">
+    <tableColumn id="5" xr3:uid="{3ACDA19A-4009-42B7-9CEC-E31BB63C9FF9}" name="Department_Name" dataDxfId="9">
       <calculatedColumnFormula>_xlfn.XLOOKUP(O2,Lookup_Departments!$A$2:$A$7,Lookup_Departments!$B$2:$B$7,"Not Found")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{DE6D60F7-3EDE-4612-8BF2-B0B2DD1F6F08}" name="Cleaned Dept_Code" dataDxfId="78">
+    <tableColumn id="6" xr3:uid="{DE6D60F7-3EDE-4612-8BF2-B0B2DD1F6F08}" name="Cleaned Dept_Code" dataDxfId="8">
       <calculatedColumnFormula>IFERROR(VLOOKUP(D2,Lookup_Departments!$A$2:$B$7,1,FALSE),"Invalid")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{EE50497A-713B-4CF0-BCF5-4B90997B9970}" name="Cleaned Hire_Date" dataDxfId="77">
+    <tableColumn id="7" xr3:uid="{EE50497A-713B-4CF0-BCF5-4B90997B9970}" name="Cleaned Hire_Date" dataDxfId="7">
       <calculatedColumnFormula>IF(ISNUMBER(E2),E2,DATE(RIGHT(E2,4),LEFT(E2,2),MID(E2,4,2)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8900855C-479F-492C-8676-F47182C8617C}" name="Year_of_Service" dataDxfId="76">
+    <tableColumn id="8" xr3:uid="{8900855C-479F-492C-8676-F47182C8617C}" name="Year_of_Service" dataDxfId="6">
       <calculatedColumnFormula>DATEDIF(P2,TODAY(),"Y")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{43DEC46E-02F9-4373-ACF7-EB3138F23FB3}" name="Cleaned Salary" dataDxfId="75">
+    <tableColumn id="9" xr3:uid="{43DEC46E-02F9-4373-ACF7-EB3138F23FB3}" name="Cleaned Salary" dataDxfId="5">
       <calculatedColumnFormula>IF(F2="",AVERAGEIF($D$2:$D$151,D2,$F$2:$F$151),F2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{ACE85FFC-D2E7-4B83-AEB3-D19D39AD1F76}" name="Cleaned Perf_Score" dataDxfId="74">
+    <tableColumn id="10" xr3:uid="{ACE85FFC-D2E7-4B83-AEB3-D19D39AD1F76}" name="Cleaned Perf_Score" dataDxfId="4">
       <calculatedColumnFormula>IF(G2="",AVERAGE($G$2:$G$158),G2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{590E8FC3-346A-46F9-9227-B1111641C818}" name="Performance_Band" dataDxfId="73">
+    <tableColumn id="11" xr3:uid="{590E8FC3-346A-46F9-9227-B1111641C818}" name="Performance_Band" dataDxfId="3">
       <calculatedColumnFormula>_xlfn.XLOOKUP(S2,Lookup_Performance!$A$2:$A$6,Lookup_Performance!$C$2:$C$6,"Not Found",-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{17C22A28-ACB1-4EA1-8590-550C4CFACB72}" name="Eligible_Bonus_Percentage" dataDxfId="70">
+    <tableColumn id="12" xr3:uid="{17C22A28-ACB1-4EA1-8590-550C4CFACB72}" name="Eligible_Bonus_Percentage" dataDxfId="2">
       <calculatedColumnFormula>_xlfn.XLOOKUP(S2,Lookup_Performance!$A$2:$A$6,Lookup_Performance!$D$2:$D$6,"Not Found",-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{599D424E-13BE-453F-ACDA-9E66433A137E}" name="Eligible_Bonus_Amount" dataDxfId="68">
+    <tableColumn id="14" xr3:uid="{599D424E-13BE-453F-ACDA-9E66433A137E}" name="Eligible_Bonus_Amount" dataDxfId="1">
       <calculatedColumnFormula>Table1[[#This Row],[Cleaned Salary]]*Table1[[#This Row],[Eligible_Bonus_Percentage]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{15000AA3-E4C9-4C52-A2F3-4B9F18A74F89}" name="Cleaned Employment_Status" dataDxfId="69">
+    <tableColumn id="13" xr3:uid="{15000AA3-E4C9-4C52-A2F3-4B9F18A74F89}" name="Cleaned Employment_Status" dataDxfId="0">
       <calculatedColumnFormula>TRIM(CLEAN(UPPER(H2)))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -22226,7 +22016,7 @@
     <col min="1" max="2" width="27.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.08984375" style="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.08984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="10.7265625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.26953125" bestFit="1" customWidth="1"/>
@@ -22629,14 +22419,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
-      <x14:slicerList>
-        <x14:slicer r:id="rId10"/>
-      </x14:slicerList>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
I modified the whole capstone project folder
</commit_message>
<xml_diff>
--- a/data/HR_Analytics_Capstone_Raw_Data.xlsx
+++ b/data/HR_Analytics_Capstone_Raw_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\IOTBTECH 2026\Excel Folder\Excel-Capstone-Project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B1FE4E-9304-4F92-9FBD-B0626924D480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07ABA0B2-ACAD-4A96-9CE4-E38859542628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2588,7 +2588,6 @@
         <c14:dropZoneFilter val="1"/>
         <c14:dropZoneCategories val="1"/>
         <c14:dropZoneData val="1"/>
-        <c14:dropZonesVisible val="1"/>
       </c14:pivotOptions>
     </c:ext>
     <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
@@ -7218,22 +7217,7 @@
     <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
     <c:pageSetup/>
   </c:printSettings>
-  <c:extLst>
-    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
-      <c14:pivotOptions>
-        <c14:dropZoneFilter val="1"/>
-        <c14:dropZoneCategories val="1"/>
-        <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
-        <c14:dropZonesVisible val="1"/>
-      </c14:pivotOptions>
-    </c:ext>
-    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
-      <c16:pivotOptions16>
-        <c16:showExpandCollapseFieldButtons val="1"/>
-      </c16:pivotOptions16>
-    </c:ext>
-  </c:extLst>
+  <c:extLst/>
 </c:chartSpace>
 </file>
 
@@ -21856,7 +21840,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{95C03F21-8440-4E60-A15F-EDE839858110}" name="Headcount &amp; Average Salary by Department" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="14" rowHeaderCaption="Department_Name">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{95C03F21-8440-4E60-A15F-EDE839858110}" name="Headcount &amp; Average Salary by Department" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16" rowHeaderCaption="Department_Name">
   <location ref="A3:C9" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField dataField="1" showAll="0"/>
@@ -22276,7 +22260,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FEAA84F8-7B84-44FD-A04F-FD9B3F7229C6}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="12" rowHeaderCaption="Employment_Status">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FEAA84F8-7B84-44FD-A04F-FD9B3F7229C6}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13" rowHeaderCaption="Employment_Status">
   <location ref="F3:G7" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -22334,7 +22318,7 @@
   <dataFields count="1">
     <dataField name="Count of Cleaned Employment_Status" fld="13" subtotal="count" baseField="12" baseItem="0"/>
   </dataFields>
-  <chartFormats count="5">
+  <chartFormats count="6">
     <chartFormat chart="7" format="9" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
@@ -22372,6 +22356,15 @@
       </pivotArea>
     </chartFormat>
     <chartFormat chart="11" format="14" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="12" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">

</xml_diff>

<commit_message>
I have completed the raedme section
</commit_message>
<xml_diff>
--- a/data/HR_Analytics_Capstone_Raw_Data.xlsx
+++ b/data/HR_Analytics_Capstone_Raw_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\IOTBTECH 2026\Excel Folder\Excel-Capstone-Project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07ABA0B2-ACAD-4A96-9CE4-E38859542628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC2B9658-63DE-485F-A20F-F82B026B3848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2613,6 +2613,666 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
+    <c:name>[HR_Analytics_Capstone_Raw_Data.xlsx]Analysis!PivotTable5</c:name>
+    <c:fmtId val="33"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1100" b="1">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:rPr>
+              <a:t>Average Salary</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-NG"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="4"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$M$17</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-NG"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$L$18:$L$23</c:f>
+              <c:strCache>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>Finance</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Human Resources</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Information Technology</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Marketing</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Operations</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$M$18:$M$23</c:f>
+              <c:numCache>
+                <c:formatCode>"₦"#,##0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>87938.5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>85649.941176470587</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>80014.258064516151</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>85508.166666666657</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>79786.666666666657</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>87282.347826086945</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-9DD9-4107-9EB9-C814B6E93C1C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="417975664"/>
+        <c:axId val="417967024"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="417975664"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-NG"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="417967024"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="417967024"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="&quot;₦&quot;#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="417975664"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="DBEEF4">
+        <a:alpha val="5098"/>
+      </a:srgbClr>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst>
+      <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+        <a:prstClr val="black">
+          <a:alpha val="40000"/>
+        </a:prstClr>
+      </a:outerShdw>
+    </a:effectLst>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-NG"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
     <c:name>[HR_Analytics_Capstone_Raw_Data.xlsx]Analysis!PivotTable3</c:name>
     <c:fmtId val="11"/>
   </c:pivotSource>
@@ -3732,7 +4392,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart12.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -8747,6 +9407,464 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[HR_Analytics_Capstone_Raw_Data.xlsx]Analysis!PivotTable8</c:name>
+    <c:fmtId val="33"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" b="1">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:rPr>
+              <a:t>Average</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" b="1" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+              </a:rPr>
+              <a:t> Tenure</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-NG"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="none"/>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="75000"/>
+                      <a:lumOff val="25000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-NG"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$F$28</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$F$29</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$F$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>6.44</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6444-4331-8ACA-6ECA3CAAD2C5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1948843487"/>
+        <c:axId val="1948855967"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1948843487"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="1948855967"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1948855967"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-NG"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1948843487"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-NG"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
       <c14:style val="103"/>
     </mc:Choice>
     <mc:Fallback>
@@ -9625,666 +10743,6 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:pivotSource>
-    <c:name>[HR_Analytics_Capstone_Raw_Data.xlsx]Analysis!PivotTable5</c:name>
-    <c:fmtId val="33"/>
-  </c:pivotSource>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1100" b="1">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              </a:rPr>
-              <a:t>Average Salary</a:t>
-            </a:r>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-NG"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:pivotFmts>
-      <c:pivotFmt>
-        <c:idx val="0"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-NG"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="1"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-NG"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="2"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-NG"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="3"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-NG"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="4"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent1"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="none"/>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-NG"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-    </c:pivotFmts>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Analysis!$M$17</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Total</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="tx1">
-                        <a:lumMod val="75000"/>
-                        <a:lumOff val="25000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-NG"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:round/>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>Analysis!$L$18:$L$23</c:f>
-              <c:strCache>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>Finance</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>Human Resources</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Information Technology</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Marketing</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Operations</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>Sales</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Analysis!$M$18:$M$23</c:f>
-              <c:numCache>
-                <c:formatCode>"₦"#,##0.00</c:formatCode>
-                <c:ptCount val="6"/>
-                <c:pt idx="0">
-                  <c:v>87938.5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>85649.941176470587</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>80014.258064516151</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>85508.166666666657</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>79786.666666666657</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>87282.347826086945</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9DD9-4107-9EB9-C814B6E93C1C}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="417975664"/>
-        <c:axId val="417967024"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="417975664"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-NG"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="417967024"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="417967024"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="1"/>
-        <c:axPos val="l"/>
-        <c:numFmt formatCode="&quot;₦&quot;#,##0.00" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="417975664"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:srgbClr val="DBEEF4">
-        <a:alpha val="5098"/>
-      </a:srgbClr>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:noFill/>
-      <a:round/>
-    </a:ln>
-    <a:effectLst>
-      <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
-        <a:prstClr val="black">
-          <a:alpha val="40000"/>
-        </a:prstClr>
-      </a:outerShdw>
-    </a:effectLst>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-NG"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-  <c:extLst>
-    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
-      <c14:pivotOptions>
-        <c14:dropZoneFilter val="1"/>
-        <c14:dropZoneCategories val="1"/>
-        <c14:dropZoneData val="1"/>
-      </c14:pivotOptions>
-    </c:ext>
-    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
-      <c16:pivotOptions16>
-        <c16:showExpandCollapseFieldButtons val="1"/>
-      </c16:pivotOptions16>
-    </c:ext>
-  </c:extLst>
-</c:chartSpace>
-</file>
-
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="23">
   <a:schemeClr val="accent3"/>
@@ -10332,6 +10790,46 @@
 </file>
 
 <file path=xl/charts/colors11.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors12.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="21">
   <a:schemeClr val="accent1"/>
 </cs:colorStyle>
@@ -10510,12 +11008,6 @@
 </file>
 
 <file path=xl/charts/colors8.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
-  <a:schemeClr val="accent1"/>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -10552,6 +11044,12 @@
     <a:lumMod val="50000"/>
     <a:lumOff val="50000"/>
   </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
+  <a:schemeClr val="accent1"/>
 </cs:colorStyle>
 </file>
 
@@ -11052,6 +11550,509 @@
 </file>
 
 <file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="205">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -11621,7 +12622,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style12.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="203">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -15362,6 +16363,509 @@
 </file>
 
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="206">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -15886,509 +17390,6 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="28575" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="75000"/>
-            <a:lumOff val="25000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -16652,6 +17653,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>179916</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>455083</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>21165</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="9" name="Chart 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0B96784-83CD-47DA-944E-1B3FF374F4FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -21772,7 +22811,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F4E7B9D-DDA8-4061-9C46-C8585D2A937B}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="30" rowHeaderCaption="">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3F4E7B9D-DDA8-4061-9C46-C8585D2A937B}" name="PivotTable8" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="34" rowHeaderCaption="">
   <location ref="F28:F29" firstHeaderRow="1" firstDataRow="1" firstDataCol="0"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -21827,6 +22866,44 @@
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
+  <chartFormats count="4">
+    <chartFormat chart="30" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="31" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="32" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="33" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">

</xml_diff>